<commit_message>
Circular 2026-033: sin la nota de firma; regla de firmas en la skill
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -3343,7 +3342,7 @@
       </c>
       <c r="M32" s="4" t="inlineStr">
         <is>
-          <t>Bonificado 6+1 cruzado. Los bonificados no suman en unidades vendidas. Falta firma de Ventas</t>
+          <t>Bonificado 6+1 cruzado. Los bonificados no suman en unidades vendidas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Circular 2026-033: enlace al PDF en Drive
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1234,8 +1234,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:M32" headerRowCount="1" totalsRowShown="0">
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N32" headerRowCount="1" totalsRowShown="0">
+  <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
     <tableColumn id="3" name="Nombre de la actividad"/>
@@ -1249,6 +1249,7 @@
     <tableColumn id="11" name="Objetivo"/>
     <tableColumn id="12" name="Resumen de la actividad"/>
     <tableColumn id="13" name="Observación"/>
+    <tableColumn id="14" name="Enlace PDF (opcional)"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1437,7 +1438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1452,6 +1453,7 @@
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="70" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="45" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="38.25" customHeight="1">
@@ -1520,6 +1522,11 @@
           <t>Observación</t>
         </is>
       </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Enlace PDF (opcional)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="51" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -1577,6 +1584,7 @@
         </is>
       </c>
       <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="n"/>
     </row>
     <row r="3" ht="51" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -1634,6 +1642,7 @@
         </is>
       </c>
       <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
     </row>
     <row r="4" ht="51" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1691,6 +1700,7 @@
         </is>
       </c>
       <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
     </row>
     <row r="5" ht="38.25" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
@@ -1748,6 +1758,7 @@
         </is>
       </c>
       <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
     </row>
     <row r="6" ht="38.25" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -1805,6 +1816,7 @@
         </is>
       </c>
       <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
     </row>
     <row r="7" ht="38.25" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
@@ -1862,6 +1874,7 @@
         </is>
       </c>
       <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
     </row>
     <row r="8" ht="51" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1919,6 +1932,7 @@
         </is>
       </c>
       <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
     </row>
     <row r="9" ht="38.25" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1976,6 +1990,7 @@
         </is>
       </c>
       <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n"/>
     </row>
     <row r="10" ht="51" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
@@ -2037,6 +2052,7 @@
           <t>Prorrogada un mes por la circular 2026-019</t>
         </is>
       </c>
+      <c r="N10" s="4" t="n"/>
     </row>
     <row r="11" ht="38.25" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
@@ -2094,6 +2110,7 @@
         </is>
       </c>
       <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="n"/>
     </row>
     <row r="12" ht="38.25" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
@@ -2151,6 +2168,7 @@
         </is>
       </c>
       <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="n"/>
     </row>
     <row r="13" ht="38.25" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2212,6 +2230,7 @@
           <t>El PDF dice año 2025 en la fecha final; se asumió 2026</t>
         </is>
       </c>
+      <c r="N13" s="4" t="n"/>
     </row>
     <row r="14" ht="38.25" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -2269,6 +2288,7 @@
         </is>
       </c>
       <c r="M14" s="4" t="n"/>
+      <c r="N14" s="4" t="n"/>
     </row>
     <row r="15" ht="38.25" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2330,6 +2350,7 @@
           <t>El PDF dice año 2025 en la fecha final; se asumió 2026</t>
         </is>
       </c>
+      <c r="N15" s="4" t="n"/>
     </row>
     <row r="16" ht="38.25" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2387,6 +2408,7 @@
         </is>
       </c>
       <c r="M16" s="4" t="n"/>
+      <c r="N16" s="4" t="n"/>
     </row>
     <row r="17" ht="38.25" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -2444,6 +2466,7 @@
         </is>
       </c>
       <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4" t="n"/>
     </row>
     <row r="18" ht="38.25" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -2505,6 +2528,7 @@
           <t>Vigencia de un solo día</t>
         </is>
       </c>
+      <c r="N18" s="4" t="n"/>
     </row>
     <row r="19" ht="38.25" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
@@ -2566,6 +2590,7 @@
         </is>
       </c>
       <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4" t="n"/>
     </row>
     <row r="20" ht="38.25" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
@@ -2627,6 +2652,7 @@
           <t>Prórroga de 2026-009</t>
         </is>
       </c>
+      <c r="N20" s="4" t="n"/>
     </row>
     <row r="21" ht="51" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
@@ -2684,6 +2710,7 @@
         </is>
       </c>
       <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="n"/>
     </row>
     <row r="22" ht="38.25" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
@@ -2745,6 +2772,7 @@
           <t>Aporte de $3.000.000 de Epithelium</t>
         </is>
       </c>
+      <c r="N22" s="4" t="n"/>
     </row>
     <row r="23" ht="38.25" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
@@ -2806,6 +2834,7 @@
           <t>Descuento 10%; NC el 28/08/2026</t>
         </is>
       </c>
+      <c r="N23" s="4" t="n"/>
     </row>
     <row r="24" ht="38.25" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
@@ -2867,6 +2896,7 @@
           <t>Descuento 15% viernes y sábado; NC el 15-16/10/2026</t>
         </is>
       </c>
+      <c r="N24" s="4" t="n"/>
     </row>
     <row r="25" ht="38.25" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
@@ -2928,6 +2958,7 @@
           <t>Meta 100 unidades; $10.000 por unidad en Protocolo Médico</t>
         </is>
       </c>
+      <c r="N25" s="4" t="n"/>
     </row>
     <row r="26" ht="38.25" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
@@ -2985,6 +3016,7 @@
         </is>
       </c>
       <c r="M26" s="4" t="n"/>
+      <c r="N26" s="4" t="n"/>
     </row>
     <row r="27" ht="38.25" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
@@ -3046,6 +3078,7 @@
           <t>$4.000 y $12.000 por unidad en Protocolo Médico</t>
         </is>
       </c>
+      <c r="N27" s="4" t="n"/>
     </row>
     <row r="28" ht="38.25" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
@@ -3107,6 +3140,7 @@
           <t>El PDF dice año 2025; se asumió 2026. Compras desde $1.500.000; 100 unidades</t>
         </is>
       </c>
+      <c r="N28" s="4" t="n"/>
     </row>
     <row r="29" ht="38.25" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
@@ -3168,6 +3202,7 @@
           <t>Bonificación 5+2 (canal 90) y 5+1 (demás)</t>
         </is>
       </c>
+      <c r="N29" s="4" t="n"/>
     </row>
     <row r="30" ht="38.25" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
@@ -3229,6 +3264,7 @@
           <t>Descuento 20%</t>
         </is>
       </c>
+      <c r="N30" s="4" t="n"/>
     </row>
     <row r="31" ht="38.25" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
@@ -3290,6 +3326,7 @@
           <t>El PDF dice año 2025; se asumió 2026. Corrige código del producto</t>
         </is>
       </c>
+      <c r="N31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -3343,6 +3380,11 @@
       <c r="M32" s="4" t="inlineStr">
         <is>
           <t>Bonificado 6+1 cruzado. Los bonificados no suman en unidades vendidas</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1M4g933hHDbjYQh2vLg3psP0dq-G2pj6O/view</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Circulares: la 2026-032 queda registrada como anulada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1234,7 +1235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N32" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N33" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1438,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N32"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3331,58 +3332,98 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2026-033</t>
+          <t>2026-032</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Codificación y colocación</t>
+          <t>Anulada</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Bonificado Cruzado</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Producto Terminado</t>
-        </is>
-      </c>
+          <t>Circular anulada</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Canales 90, 10, 11, 50, 51, 61, 70 (no aplica Bella Piel)</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>[PT0005] Sunskin Oil Free x 80 g, [PT0011] Capilplus Shampoo x 220 ml, [PT0001] Hydrafort Face x 50 g, [PT0014] Capilplus Acondicionador x 220 ml, [PT0003] Revival Crema x 50 g, [PT0012] Sensibath x 240 ml, [PT0002] Capilplus DS Shampoo Anticaspa x 220 ml, [PT0004] Hydrafort pH5 Ultrahumectante Crema x 250 g, [PT0010] Sunskin SPF 50+ Emulsión x 80 g</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="n">
-        <v>46301</v>
-      </c>
-      <c r="H32" s="5" t="n">
-        <v>46356</v>
-      </c>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="K32" s="4" t="inlineStr"/>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>La circular 2026-032 quedó anulada: no se presentó.</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Anulada. No se presentó</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>2026-033</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Codificación y colocación</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Bonificado Cruzado</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Producto Terminado</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Canales 90, 10, 11, 50, 51, 61, 70 (no aplica Bella Piel)</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>[PT0005] Sunskin Oil Free x 80 g, [PT0011] Capilplus Shampoo x 220 ml, [PT0001] Hydrafort Face x 50 g, [PT0014] Capilplus Acondicionador x 220 ml, [PT0003] Revival Crema x 50 g, [PT0012] Sensibath x 240 ml, [PT0002] Capilplus DS Shampoo Anticaspa x 220 ml, [PT0004] Hydrafort pH5 Ultrahumectante Crema x 250 g, [PT0010] Sunskin SPF 50+ Emulsión x 80 g</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>46301</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I33" s="3" t="n"/>
+      <c r="J33" s="3" t="n"/>
+      <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Impulsar la compra y codificación de los terminados de menor rotación bonificando 1 unidad de alta rotación por cada 6 compradas. Meta mensual: Sunskin Oil Free 66, Capilplus Shampoo 134, Hydrafort Face 108, Capilplus Acondicionador 42 y Revival Crema 66 uds</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L33" s="4" t="inlineStr">
         <is>
           <t>Por cada 6 uds de una referencia de baja rotación el cliente recibe 1 bonificada de alta rotación (paga solo el IVA): Sunskin Oil Free → Sensibath; Capilplus Shampoo → Capilplus DS; Hydrafort Face → Hydrafort pH5; Capilplus Acondicionador → Capilplus DS; Revival → Sunskin SPF 50+ Emulsión. Aplica por múltiplos de 6 en cada pedido, también a clientes que ya tienen el portafolio codificado. El bonificado se carga solo en Odoo.</t>
         </is>
       </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="M33" s="4" t="inlineStr">
         <is>
           <t>Bonificado 6+1 cruzado. Los bonificados no suman en unidades vendidas</t>
         </is>
       </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1M4g933hHDbjYQh2vLg3psP0dq-G2pj6O/view</t>
         </is>

</xml_diff>

<commit_message>
Circulares: se carga la 2026-034 Afilia y gana con Protocolo Medico
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1439,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3428,6 +3428,62 @@
           <t>https://drive.google.com/file/d/1M4g933hHDbjYQh2vLg3psP0dq-G2pj6O/view</t>
         </is>
       </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-034</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Incentivo Fuerza de Ventas</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Afilia y gana con Protocolo Medico</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Todo portafolio</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Canales 20, 21, 22 (Protocolo Médico)</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Todo el portafolio</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>46302</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I34" s="3" t="n"/>
+      <c r="J34" s="3" t="n"/>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>Ampliar la cobertura del Protocolo Médico: captar médicos nuevos y reactivar los de la lista (clasificación 20, 21 y 22) para que más médicos formulen cada mes</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Incentivo a la visitadora que cumpla la meta de su zona: Zona Norte y Zona Sur, 5 médicos activados o reactivados (mínimo 1 reactivado) y $249.551 cada una; Zona Desarrollo, 1 médico por activar y $100.000. Cuenta la formulación facturada de al menos $10.000 entre el 1 de septiembre y el 30 de noviembre de 2026. Se paga en diciembre con la liquidación del Protocolo Médico.</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>Anexo 1: 9 médicos por reactivar. Anexo 2: 235 por activar. Anexo 3: 29 activos (no cuentan para la meta). Los anexos no vienen en el PDF. En Zona Sur el incentivo es para Yunelis Caballero. Incluye el Formulador del Año Revival (circular 2026-001)</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circular 2026-034: quitar la nota de que los anexos no vienen en el PDF
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -3480,7 +3479,7 @@
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>Anexo 1: 9 médicos por reactivar. Anexo 2: 235 por activar. Anexo 3: 29 activos (no cuentan para la meta). Los anexos no vienen en el PDF. En Zona Sur el incentivo es para Yunelis Caballero. Incluye el Formulador del Año Revival (circular 2026-001)</t>
+          <t>Anexo 1: 9 médicos por reactivar. Anexo 2: 235 por activar. Anexo 3: 29 activos (no cuentan para la meta). En Zona Sur el incentivo es para Yunelis Caballero. Incluye el Formulador del Año Revival (circular 2026-001)</t>
         </is>
       </c>
       <c r="N34" s="4" t="n"/>

</xml_diff>

<commit_message>
Circular 2026-035: alcance a la 2026-033 (canales 70 y 90)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1438,7 +1438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3483,6 +3483,62 @@
         </is>
       </c>
       <c r="N34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>2026-035</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Alcance circular 2026-033</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Producto Terminado</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Canales 70, 90 (no aplica Bella Piel)</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>[PT0005] Sunskin Oil Free x 80 g, [PT0011] Capilplus Shampoo x 220 ml, [PT0001] Hydrafort Face x 50 g, [PT0014] Capilplus Acondicionador x 220 ml, [PT0003] Revival Crema x 50 g, [PT0012] Sensibath x 240 ml, [PT0002] Capilplus DS Shampoo Anticaspa x 220 ml, [PT0004] Hydrafort pH5 Ultrahumectante Crema x 250 g, [PT0010] Sunskin SPF 50+ Emulsión x 80 g</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I35" s="3" t="n"/>
+      <c r="J35" s="3" t="n"/>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Aclarar la circular 2026-033 Bonificado Cruzado para los canales 70 y 90: participan en la actividad, pero acceden a la bonificación adicional con la compra de los productos de baja rotación bajo su bonificado (70: 10 + 2; 90: 6 + 2)</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Alcance a la circular 2026-033: el canal 70 compra los productos de baja rotación con su bonificado 10 + 2 y, por cada 10 unidades compradas (y sus múltiplos), se bonifica 1 unidad de alta rotación del cuadro de cruces. El canal 90 compra con su bonificado 6 + 2 y, por cada 6 unidades (y sus múltiplos), se bonifica 1 unidad de alta rotación. Aplica en cada pedido que cumpla la condición. Para los canales 10, 11, 50, 51 y 61 la condición sigue igual: 6 + 1.</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Aclara 2026-033 para los canales 70 (10+2) y 90 (6+2). Los demás canales no cambian</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circular 2026-039: Bonificación Especial Queratrex Gel – Canales 20 y 90
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1234,7 +1235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N33" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N36" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1438,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3539,6 +3540,62 @@
         </is>
       </c>
       <c r="N35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-039</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Colocación</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación Especial Queratrex Gel – Canales 20 y 90</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Canales 20, 90</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>[MP0731] Queratrex Gel x 30 g</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I36" s="3" t="n"/>
+      <c r="J36" s="3" t="n"/>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>Aumentar las unidades vendidas y la recompra de Queratrex Gel x 30 g en los clientes de los canales 20 y 90, entre el 26 de octubre y el 30 de noviembre de 2026.</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación escalonada por pedido: compra 5 unidades y recibe 2 adicionales (5+2); compra 10 y recibe 5 adicionales (10+5). Bono de recompra del 10% sobre el valor de la compra de Queratrex Gel para el cliente con mínimo 2 pedidos en el periodo, reconocido con nota crédito liquidada a más tardar el 15 de diciembre de 2026. La escala se aplica por pedido (no se suman pedidos) y cuenta la fecha de inclusión del pedido, no la de entrega. Meta: Sur 3, Norte 4, Desarrollo 0, Clientes Especiales 1 (total 8).</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>Escala 5+2 y 10+5 por pedido; bono de recompra 10% con 2 o más pedidos (NC a más tardar el 15/12/2026). Sin prórroga. Los bonificados no cuentan en el bono.</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circular 2026-036: Bonificación especial de lanzamiento
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1235,7 +1235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N36" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N37" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1439,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3596,6 +3596,62 @@
         </is>
       </c>
       <c r="N36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>2026-036</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Colocación</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación especial de lanzamiento</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Canales 10, 11, 13, 14, 30, 31, 50, 51, 52, 53, 70, 71, 90</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>[MP1098] Minobit Advance Loción x 100 ml; [MP1099] Minobit Advance Loción x 60 ml; [MP1100] BimaLash Serum x 4.2 ml</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I37" s="3" t="n"/>
+      <c r="J37" s="3" t="n"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Impulsar la colocación, la codificación y la rotación de Minobit Advance Loción x 100 ml, Minobit Advance Loción x 60 ml y BimaLash Serum x 4.2 ml en los canales participantes, mediante una bonificación especial de lanzamiento 6 + 4, para aumentar su penetración y favorecer el abastecimiento inicial de los clientes.</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Por cada 6 unidades compradas de una misma referencia (y sus múltiplos), el cliente recibe 4 unidades adicionales sin costo (6 + 4): 10 unidades pagando 6, equivalente a un 40% de descuento sobre el valor de lista, adicional al descuento de tarifa del canal. Reemplaza la bonificación estándar del canal en estas referencias y no es acumulable con otras. Queda matriculada en Odoo y se asigna automáticamente en el pedido. Objetivo de codificación por zona: Sur 10, Norte 13, Desarrollo 6, Clientes Especiales 4 (total 33).</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>Bonificado 6+4 por referencia; reemplaza la bonificación estándar del canal; sin liquidación posterior.</t>
+        </is>
+      </c>
+      <c r="N37" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circulares 2026-037 y 2026-038: codificación de productos Nuevos (inicio 26 de octubre)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1235,7 +1235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N37" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N39" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1439,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3652,6 +3652,118 @@
         </is>
       </c>
       <c r="N37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-037</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Colocación</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación especial por codificación de productos Nuevos – Socios Epithelium</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Canales 20, 90</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>[MP0916] Ascorvit 20% Serum x 30 ml; [MP0734] Minobit N Espuma x 200 ml; [MP0611] Minobit TD Loción x 120 ml; [MP0586] Minobit TD Loción x 60 ml; [MP0941] Sensibath MP Syndet x 1000 ml; [MP0912] Sérum Reparador Cejas y Pestañas x 4.2 ml; [MP0750] Shampoo Anticaída con C.B.D x 250 ml; [MP0879] Syndet Niños x 220 ml</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I38" s="3" t="n"/>
+      <c r="J38" s="3" t="n"/>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Impulsar la codificación, formulación y rotación inicial de los productos Nuevo en los clientes de los canales 20 (Socio Epithelium) y 90 (Accionista con tienda de piel o punto de venta), con una bonificación 6 + 3 por única vez por cliente y producto, sin descuento adicional.</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Por cada 6 unidades compradas de un producto Nuevo, el cliente recibe 3 adicionales sin costo (6 + 3): 9 unidades pagando 6, equivalente a un 33,3% de descuento sobre el valor de lista. Aplica solo en el primer pedido en que el cliente codifica cada producto y no es acumulable con otras promociones del mismo producto. Cuenta la fecha de inclusión del pedido, no la de entrega. Queda matriculada en Odoo y se asigna automáticamente en el pedido. La meta se mide solo en el canal 90 (75% de los clientes activos, redondeado hacia arriba).</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación 6+3 única por cliente y producto. Cortes de control: 31 de octubre y 30 de noviembre.</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>2026-038</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Colocación</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Descuento especial por codificación de productos Nuevos</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Canales 10, 11, 13, 21</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>[MP0916] Ascorvit 20% Serum x 30 ml; [MP0734] Minobit N Espuma x 200 ml; [MP0611] Minobit TD Loción x 120 ml; [MP0586] Minobit TD Loción x 60 ml; [MP0941] Sensibath MP Syndet x 1000 ml; [MP0912] Sérum Reparador Cejas y Pestañas x 4.2 ml; [MP0750] Shampoo Anticaída con C.B.D x 250 ml; [MP0879] Syndet Niños x 220 ml</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Impulsar la codificación, formulación y rotación inicial de los productos Nuevo en los clientes de los canales 10, 11, 13 y 21, con una bonificación 6 + 2 por única vez por cliente y producto, sin descuento adicional.</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Por cada 6 unidades compradas de un producto Nuevo, el cliente recibe 2 adicionales sin costo (6 + 2): 8 unidades pagando 6, equivalente a un 25% de descuento sobre el valor de lista. Aplica solo en el primer pedido en que el cliente codifica cada producto y no es acumulable con otras promociones del mismo producto. Cuenta la fecha de inclusión del pedido, no la de entrega. Queda matriculada en Odoo y se asigna automáticamente en el pedido. Meta: 24 clientes a codificar (Sur 10, Norte 9, Clientes Especiales 2, Desarrollo 3).</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación 6+2 única por cliente y producto. Cortes de control: 31 de octubre y 30 de noviembre.</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circular 2026-029: Bonificación Especial Queratrex Gel (canales 10, 11, 13, 21, 50, 70 y 71)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Circulares" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Circulares" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId3"/>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="4" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1235,7 +1234,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N39" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N40" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1439,7 +1438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3764,6 +3763,62 @@
         </is>
       </c>
       <c r="N39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-029</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Colocación</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación Especial Queratrex Gel</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Canales 10, 11, 13, 21, 50, 70, 71</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>[MP0731] Queratrex Gel x 30 g</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I40" s="3" t="n"/>
+      <c r="J40" s="3" t="n"/>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>Aumentar las unidades vendidas y la recompra de Queratrex Gel x 30 g en los clientes de los canales 10, 11, 13, 21, 50, 70 y 71, entre el 26 de octubre y el 30 de noviembre de 2026.</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Bonificación escalonada por pedido: compra 5 unidades y recibe 1 adicional (5+1); compra 10 y recibe 3 adicionales (10+3). Bono de recompra del 10% sobre el valor de la compra de Queratrex Gel para el cliente con mínimo 2 pedidos en el periodo, reconocido con nota crédito liquidada a más tardar el 15 de diciembre de 2026. La escala se aplica por pedido (no se suman pedidos; rige la más alta alcanzada) y cuenta la fecha de inclusión del pedido, no la de entrega, sin prórroga. Meta de codificación: 16 clientes (Sur 6, Norte 6, Desarrollo 1, Clientes Especiales 3).</t>
+        </is>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>Escala 5+1 y 10+3 por pedido; bono de recompra 10% con 2 o más pedidos (NC a más tardar el 15/12/2026). Sin prórroga. Los bonificados no cuentan en el bono.</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circulares 2026-040 (Actividad promocional Dermatodo) y 2026-041 (Gana por codificar), dirigidas a Ciruderma S.A.S. (Dermatodo)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqBZrofp3N6yRFAotVxtJ
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -19,8 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1234,7 +1235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N40" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N42" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1438,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3819,6 +3820,118 @@
         </is>
       </c>
       <c r="N40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>2026-040</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Evacuación</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Actividad promocional Dermatodo octubre–noviembre</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Producto Terminado</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Ciruderma S.A.S. (Dermatodo)</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>[PT0002] Capilplus DS Shampoo Anticaspa x 220 ml; [PT0012] Sensibath x 240 ml; [PT0014] Capilplus Acondicionador x 220 ml; [PT0011] Capilplus Shampoo x 220 ml</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>46321</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I41" s="3" t="n"/>
+      <c r="J41" s="3" t="n"/>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Apoyar a Dermatodo (Ciruderma S.A.S.) en su campaña de descuentos de la última semana de octubre y el mes de noviembre de 2026, para impulsar la evacuación de inventario y la rotación de los productos relacionados, en sus puntos de venta físicos y canales digitales. Meta: evacuar 90 unidades entre el 26 de octubre y el 30 de noviembre de 2026: Capilplus DS Shampoo Anticaspa x 220 ml (24), Sensibath x 240 ml (30), Capilplus Acondicionador x 220 ml (12) y Capilplus Shampoo x 220 ml (24).</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Descuento del 10% sobre el valor de venta Epithelium antes de IVA, del 26 de octubre al 30 de noviembre de 2026, en puntos de venta físicos y canales digitales de Dermatodo. Aplica solo a los 4 productos terminados de la circular y no es acumulable con otras promociones sobre los mismos productos. El cliente envía la relación de ventas POS a más tardar el 6 de diciembre de 2026; la liquidación es por nota crédito, emitida entre el 9 y el 16 de diciembre de 2026, una vez validadas las ventas efectivas.</t>
+        </is>
+      </c>
+      <c r="M41" s="4" t="inlineStr">
+        <is>
+          <t>Descuento 10% antes de IVA; meta 90 unidades; ventas POS del cliente a más tardar el 6/12/2026; NC entre el 9 y el 16/12/2026.</t>
+        </is>
+      </c>
+      <c r="N41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-041</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Codificación</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Gana por codificar</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Producto Terminado</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Ciruderma S.A.S. (Dermatodo)</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>[PT0001] Hydrafort Face x 50 g; [PT0003] Revival Crema x 50 g; [PT0004] Hydrafort pH5 Ultrahumectante Crema x 250 g; [PT0005] Sunskin Oil Free x 80 g; [PT0009] Sunskin SPF 50+ Gel x 80 g; [PT0010] Sunskin SPF 50+ Emulsión x 80 g</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="n">
+        <v>46327</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>46356</v>
+      </c>
+      <c r="I42" s="3" t="n"/>
+      <c r="J42" s="3" t="n"/>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>Codificar toda la línea de producto terminado pendiente (6 referencias de Sunskin, Hydrafort y Revival) en Ciruderma S.A.S. (Dermatodo) durante noviembre, con un 20% de descuento adicional antes de IVA, para que los productos queden disponibles para la temporada de vacaciones y cierre de año. Meta: 6 de 6 referencias codificadas.</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Durante noviembre, Dermatodo obtiene un 20% de descuento adicional, antes de IVA, en cada referencia que codifique, producto por producto, con un único pedido de codificación de mínimo 6 unidades por referencia (cuenta la fecha de inclusión del pedido). Aplica solo a las 6 referencias de la circular y no a unidades bonificadas. La circular 2026-033 Bonificado Cruzado no aplica para Ciruderma en estos productos: el visitador médico comercial debe garantizar que no se aplique al hacer el pedido. El descuento queda matriculado en Odoo y se refleja en la factura (sin nota crédito).</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>Pedido único de codificación, mínimo 6 unidades por referencia; 20% adicional antes de IVA; no aplica 2026-033 (Bonificado Cruzado) para Ciruderma en estos productos; sin nota crédito.</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circular 2026-042: Parrilla Promocional noviembre-enero (desde el 3 de noviembre)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017DU2f1u7EwZqAFVEwrSBRs
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Circulares" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Circulares" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="4" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -1235,7 +1235,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N42" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N43" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1439,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3932,6 +3932,62 @@
         </is>
       </c>
       <c r="N42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-042</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Evacuación</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Parrilla Promocional. Noviembre - Enero</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido / Producto Terminado</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Canales 20, 21, 22</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>[MP0586] Minobit TD Loción x 60 ml; [MP0611] Minobit TD Loción x 120 ml; [MP0916] Ascorvit 20% Serum x 30 ml; [MP0750] Shampoo Anticaída con C.B.D. x 250 ml; [PT0014] Capilplus Acondicionador x 220 ml; [PT0001] Hydrafort Face x 50 g; [PT0003] Revival Crema x 50 g</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>46329</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>46418</v>
+      </c>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>Presentar la parrilla promocional al 100% del panel médico de cada zona, con mínimo 1 impacto mensual</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Parrilla noviembre-enero para canales 20, 21 y 22: Minobit TD Loción, Ascorvit 20% Serum, Shampoo Anticaída con C.B.D., Capilplus Acondicionador, Hydrafort Face y Revival Crema. Visita mensual (presencial en Bogotá, virtual en regiones), refuerzo semanal y mensaje unificado.</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Continúa la parrilla de la circular 2026-025</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>

<commit_message>
Circular 2026-042: vigencia del 1 de noviembre de 2026 al 31 de enero de 2027, como dice la circular
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017DU2f1u7EwZqAFVEwrSBRs
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -19,9 +19,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -3965,7 +3964,7 @@
         </is>
       </c>
       <c r="G43" s="5" t="n">
-        <v>46329</v>
+        <v>46327</v>
       </c>
       <c r="H43" s="5" t="n">
         <v>46418</v>

</xml_diff>

<commit_message>
Circular 2026-042: Parrilla Promocional noviembre - enero (#11)
* Circular 2026-042: Parrilla Promocional noviembre-enero (desde el 3 de noviembre)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017DU2f1u7EwZqAFVEwrSBRs

* Circular 2026-042: vigencia del 1 de noviembre de 2026 al 31 de enero de 2027, como dice la circular

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017DU2f1u7EwZqAFVEwrSBRs

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/Circulares.xlsx
+++ b/datos/Circulares.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Circulares" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Circulares" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="4" r:id="rId3"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -1235,7 +1234,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N42" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Circulares" displayName="Circulares" ref="A1:N43" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="14">
     <tableColumn id="1" name="Circular"/>
     <tableColumn id="2" name="Tipo"/>
@@ -1439,7 +1438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3932,6 +3931,62 @@
         </is>
       </c>
       <c r="N42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2026-042</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Evacuación</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Parrilla Promocional. Noviembre - Enero</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Magistral de Pedido / Producto Terminado</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Canales 20, 21, 22</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>[MP0586] Minobit TD Loción x 60 ml; [MP0611] Minobit TD Loción x 120 ml; [MP0916] Ascorvit 20% Serum x 30 ml; [MP0750] Shampoo Anticaída con C.B.D. x 250 ml; [PT0014] Capilplus Acondicionador x 220 ml; [PT0001] Hydrafort Face x 50 g; [PT0003] Revival Crema x 50 g</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>46327</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>46418</v>
+      </c>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="3" t="n"/>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>Presentar la parrilla promocional al 100% del panel médico de cada zona, con mínimo 1 impacto mensual</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Parrilla noviembre-enero para canales 20, 21 y 22: Minobit TD Loción, Ascorvit 20% Serum, Shampoo Anticaída con C.B.D., Capilplus Acondicionador, Hydrafort Face y Revival Crema. Visita mensual (presencial en Bogotá, virtual en regiones), refuerzo semanal y mensaje unificado.</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>Continúa la parrilla de la circular 2026-025</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="n"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:M31">

</xml_diff>